<commit_message>
feat: categorize car features, remove old detail-copy fields
CarFeature now has a category (Exterior / Interior / Performance /
Audio and Communications) chosen via admin dropdown instead of the
front-end guessing it from free text. /api/cars/:id/ features now
returns [{category, text}, ...].

Adds categorize_features command to best-effort categorize existing
free-text features by keyword — dealers should review/correct the
results in the admin.

Removes Car.summary/performance/interior/safety (the old "Car
Specification" accordion copy) and the details serializer field —
superseded by categorized features per the front-end redesign.
</commit_message>
<xml_diff>
--- a/docs/car_import_template.xlsx
+++ b/docs/car_import_template.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB2"/>
+  <dimension ref="A1:X2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -442,13 +442,9 @@
     <col width="18" customWidth="1" min="19" max="19"/>
     <col width="15" customWidth="1" min="20" max="20"/>
     <col width="14" customWidth="1" min="21" max="21"/>
-    <col width="15" customWidth="1" min="22" max="22"/>
-    <col width="14" customWidth="1" min="23" max="23"/>
+    <col width="17" customWidth="1" min="22" max="22"/>
+    <col width="20" customWidth="1" min="23" max="23"/>
     <col width="14" customWidth="1" min="24" max="24"/>
-    <col width="14" customWidth="1" min="25" max="25"/>
-    <col width="17" customWidth="1" min="26" max="26"/>
-    <col width="20" customWidth="1" min="27" max="27"/>
-    <col width="14" customWidth="1" min="28" max="28"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -554,40 +550,20 @@
       </c>
       <c r="U1" s="1" t="inlineStr">
         <is>
-          <t>summary</t>
+          <t>video_url</t>
         </is>
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
-          <t>performance</t>
+          <t>location_name</t>
         </is>
       </c>
       <c r="W1" s="1" t="inlineStr">
         <is>
-          <t>interior</t>
+          <t>location_address</t>
         </is>
       </c>
       <c r="X1" s="1" t="inlineStr">
-        <is>
-          <t>safety</t>
-        </is>
-      </c>
-      <c r="Y1" s="1" t="inlineStr">
-        <is>
-          <t>video_url</t>
-        </is>
-      </c>
-      <c r="Z1" s="1" t="inlineStr">
-        <is>
-          <t>location_name</t>
-        </is>
-      </c>
-      <c r="AA1" s="1" t="inlineStr">
-        <is>
-          <t>location_address</t>
-        </is>
-      </c>
-      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
@@ -678,30 +654,10 @@
           <t>A well-maintained 3 Series in excellent condition.</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>Full service history, 1 owner.</t>
-        </is>
-      </c>
-      <c r="V2" t="inlineStr">
-        <is>
-          <t>320d engine, ~50mpg combined.</t>
-        </is>
-      </c>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>Leather seats, heated front seats.</t>
-        </is>
-      </c>
+      <c r="U2" t="inlineStr"/>
+      <c r="V2" t="inlineStr"/>
+      <c r="W2" t="inlineStr"/>
       <c r="X2" t="inlineStr">
-        <is>
-          <t>6 airbags, ABS, ESP.</t>
-        </is>
-      </c>
-      <c r="Y2" t="inlineStr"/>
-      <c r="Z2" t="inlineStr"/>
-      <c r="AA2" t="inlineStr"/>
-      <c r="AB2" t="inlineStr">
         <is>
           <t>available</t>
         </is>

</xml_diff>